<commit_message>
Correct Lead 170 status to technical qualification passed and regenerate reports
</commit_message>
<xml_diff>
--- a/costing-report-2026-10-01-updated.xlsx
+++ b/costing-report-2026-10-01-updated.xlsx
@@ -5446,10 +5446,10 @@
         <v>241</v>
       </c>
       <c r="F110" t="s">
-        <v>304</v>
+        <v>308</v>
       </c>
       <c r="G110">
-        <v>3580807</v>
+        <v>5563501</v>
       </c>
       <c r="H110" t="s">
         <v>310</v>

</xml_diff>